<commit_message>
Week 2: annual report RAG, research agent filing analyst, web UI
- RAG: cninfo annual report download, section-aware chunking with page ranges,
  bge-m3 + Milvus Lite and jieba BM25 hybrid retrieval, RRF, bge-reranker, query
  rewrite + HyDE, page-cited answers with citation/number verification and one rewrite
- Eval set (20 questions, Midea 2025 annual report): hybrid + rerank Hit@5 95% vs
  dense-only 80%; end-to-end accuracy 20/20 with all checks passing
- Research agent: filing-analyst sub-agent, annual report search tool for the
  financial analyst, progress events; serialize MPS inference (Metal crash under
  concurrent sub-agent searches)
- Web: FastAPI with background jobs + SSE, Vue 3 pages for risk, research, filings Q&A
- Fixes: PDF line joining no longer glues table cells; header detection on short docs
- 25 tests

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/samples/000333_DCF模型.xlsx
+++ b/docs/samples/000333_DCF模型.xlsx
@@ -549,7 +549,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>取近 3 年均值 16.4%（2023-2025：16.2%/17.0%/16.1%）</t>
+          <t>近3年均值16.4%[E15]，与2025年16.1%接近</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>取近 3 年均值 2.0%，与 6 年区间 1.8%-2.0% 一致</t>
+          <t>近3年均值2.0%[E15]</t>
         </is>
       </c>
     </row>
@@ -579,7 +579,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>取近 3 年均值 2.0%（2023-2025：1.7%/1.9%/2.4%）</t>
+          <t>近3年均值2.0%[E15]，2025年2.4%略高，取均值</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>营运资本比率波动大（-12.5% 至 +8.1%），按规则取近 3 年均值 -3.2%</t>
+          <t>近3年均值-3.2%[E15]；2025年8.1%为异常跳升，不采用</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CAPM 参考 WACC 6.45%（rf 1.65%、Blume 调整 Beta 0.87、ERP 6%、税后债务成本 2.41%、股权权重 90.7%）</t>
+          <t>工具CAPM计算6.45%[E17]：rf 1.65%+β0.87×ERP6%=Ke 6.87%，税后债务成本2.41%，E/D权重90.69%/9.31%</t>
         </is>
       </c>
     </row>
@@ -624,7 +624,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.5%，低于 3% 上限，考虑家电行业成熟期名义增长</t>
+          <t>2.5%，低于3%上限，参考长期名义GDP与家电行业成熟期增速</t>
         </is>
       </c>
     </row>
@@ -769,13 +769,13 @@
         <v>0.06</v>
       </c>
       <c r="D4" s="5" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="E4" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="E4" s="5" t="n">
+      <c r="F4" s="5" t="n">
         <v>0.045</v>
-      </c>
-      <c r="F4" s="5" t="n">
-        <v>0.04</v>
       </c>
     </row>
     <row r="5">
@@ -785,19 +785,19 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>0.1</v>
+        <v>0.102</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>0.1</v>
+        <v>0.102</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>0.1</v>
+        <v>0.102</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.1</v>
+        <v>0.102</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1</v>
+        <v>0.102</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Cross-validate against FinanceToolkit and empyrical; earnings-quality review; nine-chapter memo
- tests/test_cross_validation.py: DCF, two-stage DDM, PB-ROE vs Gordon, CAPM, DuPont, Altman Z,
  Piotroski criteria vs FinanceToolkit; VaR/CVaR/max drawdown/volatility/beta vs empyrical
- valuation/quality.py: DuPont (3/5-step), Piotroski F, Altman Z / Z'', Beneish M, accruals,
  rule-based A-D earnings credibility grade; reverse DCF (market-implied growth)
- Research memo restructured after equity-research-skill: one-page summary with expectations-gap
  table, earnings-quality review before valuation, counter-case and pre-mortem; completeness check
- Fixes: explicit cash semantics for extra cash, 8K output limit for the lead agent
- 48 tests

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/samples/000333_DCF模型.xlsx
+++ b/docs/samples/000333_DCF模型.xlsx
@@ -75,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -85,6 +85,7 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -456,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -530,7 +531,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>-146.72077024</v>
+        <v>-582.2980568900001</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -549,7 +550,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>近3年均值16.4%[E15]，与2025年16.1%接近</t>
+          <t>取近3年均值16.4%（2023 16.2%/2024 17.0%/2025 16.1%，E16）</t>
         </is>
       </c>
     </row>
@@ -564,7 +565,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>近3年均值2.0%[E15]</t>
+          <t>取近3年均值2.0%（E16），2020-2025区间1.8%-2.0%</t>
         </is>
       </c>
     </row>
@@ -579,7 +580,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>近3年均值2.0%[E15]，2025年2.4%略高，取均值</t>
+          <t>取近3年均值2.0%（E16），2025年2.4%略高，行业产能利用率不足六成下不假设扩产</t>
         </is>
       </c>
     </row>
@@ -590,11 +591,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>-0.032</v>
+        <v>-0.127</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>近3年均值-3.2%[E15]；2025年8.1%为异常跳升，不采用</t>
+          <t>取近3年均值-12.7%（2023 -11.8%/2024 -12.9%/2025 -13.5%，E16），波动区间-8.2%~-13.5%，负营运资本为渠道占款特征</t>
         </is>
       </c>
     </row>
@@ -609,7 +610,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>工具CAPM计算6.45%[E17]：rf 1.65%+β0.87×ERP6%=Ke 6.87%，税后债务成本2.41%，E/D权重90.69%/9.31%</t>
+          <t>CAPM计算值6.45%（E17）：rf 1.65%、Beta 0.87（Blume调整）、ERP 6%、税后债务成本2.41%、E/V 90.69%</t>
         </is>
       </c>
     </row>
@@ -624,7 +625,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.5%，低于3%上限，参考长期名义GDP与家电行业成熟期增速</t>
+          <t>取2.5%，低于3%上限；家电行业成熟期，长期增速参考通胀+份额提升</t>
         </is>
       </c>
     </row>
@@ -682,6 +683,32 @@
         <v>86.54000000000001</v>
       </c>
       <c r="C17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>其他类现金资产（需年报佐证）</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>保守情形填0：其他类现金资产2418.4亿元（E16）虽经年报附注确认为定期存款/固定收益类产品（E18/E19），但本情景按用户要求保守不计入</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>汇率：报表币种 → 股价币种</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -735,7 +762,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>期数 t</t>
         </is>
@@ -757,29 +784,29 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>收入增速</t>
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>0.055</v>
+        <v>0.045</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.045</v>
+        <v>0.035</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>EBIT 利润率</t>
         </is>
@@ -801,271 +828,271 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>营业总收入</t>
         </is>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="9">
         <f>假设!$B$5*(1+B4)</f>
         <v/>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="9">
         <f>B6*(1+C4)</f>
         <v/>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="9">
         <f>C6*(1+D4)</f>
         <v/>
       </c>
-      <c r="E6" s="8">
+      <c r="E6" s="9">
         <f>D6*(1+E4)</f>
         <v/>
       </c>
-      <c r="F6" s="8">
+      <c r="F6" s="9">
         <f>E6*(1+F4)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>EBIT</t>
         </is>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="9">
         <f>B6*B5</f>
         <v/>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="9">
         <f>C6*C5</f>
         <v/>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="9">
         <f>D6*D5</f>
         <v/>
       </c>
-      <c r="E7" s="8">
+      <c r="E7" s="9">
         <f>E6*E5</f>
         <v/>
       </c>
-      <c r="F7" s="8">
+      <c r="F7" s="9">
         <f>F6*F5</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>NOPAT = EBIT×(1−税率)</t>
         </is>
       </c>
-      <c r="B8" s="8">
+      <c r="B8" s="9">
         <f>B7*(1-假设!$B$7)</f>
         <v/>
       </c>
-      <c r="C8" s="8">
+      <c r="C8" s="9">
         <f>C7*(1-假设!$B$7)</f>
         <v/>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="9">
         <f>D7*(1-假设!$B$7)</f>
         <v/>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="9">
         <f>E7*(1-假设!$B$7)</f>
         <v/>
       </c>
-      <c r="F8" s="8">
+      <c r="F8" s="9">
         <f>F7*(1-假设!$B$7)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>折旧摊销</t>
         </is>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="9">
         <f>B6*假设!$B$8</f>
         <v/>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="9">
         <f>C6*假设!$B$8</f>
         <v/>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="9">
         <f>D6*假设!$B$8</f>
         <v/>
       </c>
-      <c r="E9" s="8">
+      <c r="E9" s="9">
         <f>E6*假设!$B$8</f>
         <v/>
       </c>
-      <c r="F9" s="8">
+      <c r="F9" s="9">
         <f>F6*假设!$B$8</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>资本开支</t>
         </is>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="9">
         <f>B6*假设!$B$9</f>
         <v/>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="9">
         <f>C6*假设!$B$9</f>
         <v/>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="9">
         <f>D6*假设!$B$9</f>
         <v/>
       </c>
-      <c r="E10" s="8">
+      <c r="E10" s="9">
         <f>E6*假设!$B$9</f>
         <v/>
       </c>
-      <c r="F10" s="8">
+      <c r="F10" s="9">
         <f>F6*假设!$B$9</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>经营性营运资本</t>
         </is>
       </c>
-      <c r="B11" s="8">
+      <c r="B11" s="9">
         <f>B6*假设!$B$10</f>
         <v/>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="9">
         <f>C6*假设!$B$10</f>
         <v/>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="9">
         <f>D6*假设!$B$10</f>
         <v/>
       </c>
-      <c r="E11" s="8">
+      <c r="E11" s="9">
         <f>E6*假设!$B$10</f>
         <v/>
       </c>
-      <c r="F11" s="8">
+      <c r="F11" s="9">
         <f>F6*假设!$B$10</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>营运资本变动 ΔNWC</t>
         </is>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="9">
         <f>B11-假设!$B$6</f>
         <v/>
       </c>
-      <c r="C12" s="8">
+      <c r="C12" s="9">
         <f>C11-B11</f>
         <v/>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="9">
         <f>D11-C11</f>
         <v/>
       </c>
-      <c r="E12" s="8">
+      <c r="E12" s="9">
         <f>E11-D11</f>
         <v/>
       </c>
-      <c r="F12" s="8">
+      <c r="F12" s="9">
         <f>F11-E11</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>FCFF</t>
         </is>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="9">
         <f>B8+B9-B10-B12</f>
         <v/>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="9">
         <f>C8+C9-C10-C12</f>
         <v/>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="9">
         <f>D8+D9-D10-D12</f>
         <v/>
       </c>
-      <c r="E13" s="8">
+      <c r="E13" s="9">
         <f>E8+E9-E10-E12</f>
         <v/>
       </c>
-      <c r="F13" s="8">
+      <c r="F13" s="9">
         <f>F8+F9-F10-F12</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>折现因子</t>
         </is>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="11">
         <f>1/(1+假设!$B$11)^B3</f>
         <v/>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="11">
         <f>1/(1+假设!$B$11)^C3</f>
         <v/>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="11">
         <f>1/(1+假设!$B$11)^D3</f>
         <v/>
       </c>
-      <c r="E14" s="10">
+      <c r="E14" s="11">
         <f>1/(1+假设!$B$11)^E3</f>
         <v/>
       </c>
-      <c r="F14" s="10">
+      <c r="F14" s="11">
         <f>1/(1+假设!$B$11)^F3</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>FCFF 现值</t>
         </is>
       </c>
-      <c r="B15" s="8">
+      <c r="B15" s="9">
         <f>B13*B14</f>
         <v/>
       </c>
-      <c r="C15" s="8">
+      <c r="C15" s="9">
         <f>C13*C14</f>
         <v/>
       </c>
-      <c r="D15" s="8">
+      <c r="D15" s="9">
         <f>D13*D14</f>
         <v/>
       </c>
-      <c r="E15" s="8">
+      <c r="E15" s="9">
         <f>E13*E14</f>
         <v/>
       </c>
-      <c r="F15" s="8">
+      <c r="F15" s="9">
         <f>F13*F14</f>
         <v/>
       </c>
@@ -1096,133 +1123,133 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>预测期 FCFF 现值合计</t>
         </is>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="9">
         <f>SUM(预测!B15:F15)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>终值（戈登增长）</t>
         </is>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="9">
         <f>预测!F13*(1+假设!B12)/(假设!B11-假设!B12)</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>终值现值</t>
         </is>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="9">
         <f>B4/(1+假设!B11)^5</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>企业价值 EV</t>
         </is>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="9">
         <f>B3+B5</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>减：有息负债</t>
         </is>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="9">
         <f>假设!B13</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>加：现金</t>
-        </is>
-      </c>
-      <c r="B8" s="8">
-        <f>假设!B14</f>
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>加：现金（含其他类现金资产）</t>
+        </is>
+      </c>
+      <c r="B8" s="9">
+        <f>假设!B14+假设!B18</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>减：少数股东权益</t>
         </is>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="9">
         <f>假设!B15</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>股权价值</t>
         </is>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="9">
         <f>B6-B7+B8-B9</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>每股价值（元）</t>
-        </is>
-      </c>
-      <c r="B11" s="11">
-        <f>B10/假设!B16</f>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>每股价值（股价币种）</t>
+        </is>
+      </c>
+      <c r="B11" s="12">
+        <f>B10/假设!B16*假设!B19</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>当前股价（元）</t>
-        </is>
-      </c>
-      <c r="B12" s="11">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>当前股价</t>
+        </is>
+      </c>
+      <c r="B12" s="12">
         <f>假设!B17</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>相对现价</t>
         </is>
       </c>
-      <c r="B13" s="12">
+      <c r="B13" s="13">
         <f>B11/B12-1</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>终值占 EV 比重</t>
         </is>
       </c>
-      <c r="B14" s="12">
+      <c r="B14" s="13">
         <f>B5/B6</f>
         <v/>
       </c>
@@ -1277,24 +1304,24 @@
       <c r="A5" s="5" t="n">
         <v>0.0545</v>
       </c>
-      <c r="B5" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A5)^预测!$B$3:$F$3)+预测!$F$13*(1+B$4)/($A5-B$4)/(1+$A5)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
-        <v/>
-      </c>
-      <c r="C5" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A5)^预测!$B$3:$F$3)+预测!$F$13*(1+C$4)/($A5-C$4)/(1+$A5)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
-        <v/>
-      </c>
-      <c r="D5" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A5)^预测!$B$3:$F$3)+预测!$F$13*(1+D$4)/($A5-D$4)/(1+$A5)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
-        <v/>
-      </c>
-      <c r="E5" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A5)^预测!$B$3:$F$3)+预测!$F$13*(1+E$4)/($A5-E$4)/(1+$A5)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
-        <v/>
-      </c>
-      <c r="F5" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A5)^预测!$B$3:$F$3)+预测!$F$13*(1+F$4)/($A5-F$4)/(1+$A5)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
+      <c r="B5" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A5)^预测!$B$3:$F$3)+预测!$F$13*(1+B$4)/($A5-B$4)/(1+$A5)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
+        <v/>
+      </c>
+      <c r="C5" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A5)^预测!$B$3:$F$3)+预测!$F$13*(1+C$4)/($A5-C$4)/(1+$A5)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
+        <v/>
+      </c>
+      <c r="D5" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A5)^预测!$B$3:$F$3)+预测!$F$13*(1+D$4)/($A5-D$4)/(1+$A5)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
+        <v/>
+      </c>
+      <c r="E5" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A5)^预测!$B$3:$F$3)+预测!$F$13*(1+E$4)/($A5-E$4)/(1+$A5)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
+        <v/>
+      </c>
+      <c r="F5" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A5)^预测!$B$3:$F$3)+预测!$F$13*(1+F$4)/($A5-F$4)/(1+$A5)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
         <v/>
       </c>
     </row>
@@ -1302,24 +1329,24 @@
       <c r="A6" s="5" t="n">
         <v>0.0595</v>
       </c>
-      <c r="B6" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A6)^预测!$B$3:$F$3)+预测!$F$13*(1+B$4)/($A6-B$4)/(1+$A6)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
-        <v/>
-      </c>
-      <c r="C6" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A6)^预测!$B$3:$F$3)+预测!$F$13*(1+C$4)/($A6-C$4)/(1+$A6)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
-        <v/>
-      </c>
-      <c r="D6" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A6)^预测!$B$3:$F$3)+预测!$F$13*(1+D$4)/($A6-D$4)/(1+$A6)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
-        <v/>
-      </c>
-      <c r="E6" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A6)^预测!$B$3:$F$3)+预测!$F$13*(1+E$4)/($A6-E$4)/(1+$A6)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
-        <v/>
-      </c>
-      <c r="F6" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A6)^预测!$B$3:$F$3)+预测!$F$13*(1+F$4)/($A6-F$4)/(1+$A6)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
+      <c r="B6" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A6)^预测!$B$3:$F$3)+预测!$F$13*(1+B$4)/($A6-B$4)/(1+$A6)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
+        <v/>
+      </c>
+      <c r="C6" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A6)^预测!$B$3:$F$3)+预测!$F$13*(1+C$4)/($A6-C$4)/(1+$A6)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
+        <v/>
+      </c>
+      <c r="D6" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A6)^预测!$B$3:$F$3)+预测!$F$13*(1+D$4)/($A6-D$4)/(1+$A6)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
+        <v/>
+      </c>
+      <c r="E6" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A6)^预测!$B$3:$F$3)+预测!$F$13*(1+E$4)/($A6-E$4)/(1+$A6)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
+        <v/>
+      </c>
+      <c r="F6" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A6)^预测!$B$3:$F$3)+预测!$F$13*(1+F$4)/($A6-F$4)/(1+$A6)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
         <v/>
       </c>
     </row>
@@ -1327,24 +1354,24 @@
       <c r="A7" s="5" t="n">
         <v>0.0645</v>
       </c>
-      <c r="B7" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A7)^预测!$B$3:$F$3)+预测!$F$13*(1+B$4)/($A7-B$4)/(1+$A7)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
-        <v/>
-      </c>
-      <c r="C7" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A7)^预测!$B$3:$F$3)+预测!$F$13*(1+C$4)/($A7-C$4)/(1+$A7)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
-        <v/>
-      </c>
-      <c r="D7" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A7)^预测!$B$3:$F$3)+预测!$F$13*(1+D$4)/($A7-D$4)/(1+$A7)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
-        <v/>
-      </c>
-      <c r="E7" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A7)^预测!$B$3:$F$3)+预测!$F$13*(1+E$4)/($A7-E$4)/(1+$A7)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
-        <v/>
-      </c>
-      <c r="F7" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A7)^预测!$B$3:$F$3)+预测!$F$13*(1+F$4)/($A7-F$4)/(1+$A7)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
+      <c r="B7" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A7)^预测!$B$3:$F$3)+预测!$F$13*(1+B$4)/($A7-B$4)/(1+$A7)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
+        <v/>
+      </c>
+      <c r="C7" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A7)^预测!$B$3:$F$3)+预测!$F$13*(1+C$4)/($A7-C$4)/(1+$A7)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
+        <v/>
+      </c>
+      <c r="D7" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A7)^预测!$B$3:$F$3)+预测!$F$13*(1+D$4)/($A7-D$4)/(1+$A7)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
+        <v/>
+      </c>
+      <c r="E7" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A7)^预测!$B$3:$F$3)+预测!$F$13*(1+E$4)/($A7-E$4)/(1+$A7)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
+        <v/>
+      </c>
+      <c r="F7" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A7)^预测!$B$3:$F$3)+预测!$F$13*(1+F$4)/($A7-F$4)/(1+$A7)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
         <v/>
       </c>
     </row>
@@ -1352,24 +1379,24 @@
       <c r="A8" s="5" t="n">
         <v>0.06950000000000001</v>
       </c>
-      <c r="B8" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A8)^预测!$B$3:$F$3)+预测!$F$13*(1+B$4)/($A8-B$4)/(1+$A8)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
-        <v/>
-      </c>
-      <c r="C8" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A8)^预测!$B$3:$F$3)+预测!$F$13*(1+C$4)/($A8-C$4)/(1+$A8)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
-        <v/>
-      </c>
-      <c r="D8" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A8)^预测!$B$3:$F$3)+预测!$F$13*(1+D$4)/($A8-D$4)/(1+$A8)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
-        <v/>
-      </c>
-      <c r="E8" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A8)^预测!$B$3:$F$3)+预测!$F$13*(1+E$4)/($A8-E$4)/(1+$A8)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
-        <v/>
-      </c>
-      <c r="F8" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A8)^预测!$B$3:$F$3)+预测!$F$13*(1+F$4)/($A8-F$4)/(1+$A8)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
+      <c r="B8" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A8)^预测!$B$3:$F$3)+预测!$F$13*(1+B$4)/($A8-B$4)/(1+$A8)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
+        <v/>
+      </c>
+      <c r="C8" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A8)^预测!$B$3:$F$3)+预测!$F$13*(1+C$4)/($A8-C$4)/(1+$A8)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
+        <v/>
+      </c>
+      <c r="D8" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A8)^预测!$B$3:$F$3)+预测!$F$13*(1+D$4)/($A8-D$4)/(1+$A8)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
+        <v/>
+      </c>
+      <c r="E8" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A8)^预测!$B$3:$F$3)+预测!$F$13*(1+E$4)/($A8-E$4)/(1+$A8)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
+        <v/>
+      </c>
+      <c r="F8" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A8)^预测!$B$3:$F$3)+预测!$F$13*(1+F$4)/($A8-F$4)/(1+$A8)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
         <v/>
       </c>
     </row>
@@ -1377,24 +1404,24 @@
       <c r="A9" s="5" t="n">
         <v>0.0745</v>
       </c>
-      <c r="B9" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A9)^预测!$B$3:$F$3)+预测!$F$13*(1+B$4)/($A9-B$4)/(1+$A9)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
-        <v/>
-      </c>
-      <c r="C9" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A9)^预测!$B$3:$F$3)+预测!$F$13*(1+C$4)/($A9-C$4)/(1+$A9)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
-        <v/>
-      </c>
-      <c r="D9" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A9)^预测!$B$3:$F$3)+预测!$F$13*(1+D$4)/($A9-D$4)/(1+$A9)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
-        <v/>
-      </c>
-      <c r="E9" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A9)^预测!$B$3:$F$3)+预测!$F$13*(1+E$4)/($A9-E$4)/(1+$A9)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
-        <v/>
-      </c>
-      <c r="F9" s="11">
-        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A9)^预测!$B$3:$F$3)+预测!$F$13*(1+F$4)/($A9-F$4)/(1+$A9)^5-假设!$B$13+假设!$B$14-假设!$B$15)/假设!$B$16</f>
+      <c r="B9" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A9)^预测!$B$3:$F$3)+预测!$F$13*(1+B$4)/($A9-B$4)/(1+$A9)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
+        <v/>
+      </c>
+      <c r="C9" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A9)^预测!$B$3:$F$3)+预测!$F$13*(1+C$4)/($A9-C$4)/(1+$A9)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
+        <v/>
+      </c>
+      <c r="D9" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A9)^预测!$B$3:$F$3)+预测!$F$13*(1+D$4)/($A9-D$4)/(1+$A9)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
+        <v/>
+      </c>
+      <c r="E9" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A9)^预测!$B$3:$F$3)+预测!$F$13*(1+E$4)/($A9-E$4)/(1+$A9)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
+        <v/>
+      </c>
+      <c r="F9" s="12">
+        <f>(SUMPRODUCT(预测!$B$13:$F$13/(1+$A9)^预测!$B$3:$F$3)+预测!$F$13*(1+F$4)/($A9-F$4)/(1+$A9)^5-假设!$B$13+假设!$B$14+假设!$B$18-假设!$B$15)/假设!$B$16*假设!$B$19</f>
         <v/>
       </c>
     </row>
@@ -1493,56 +1520,56 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>股权成本 = rf + β×ERP</t>
         </is>
       </c>
-      <c r="B10" s="12">
+      <c r="B10" s="13">
         <f>B3+B4*B5</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>税后债务成本</t>
         </is>
       </c>
-      <c r="B11" s="12">
+      <c r="B11" s="13">
         <f>B6*(1-B7)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>股权权重</t>
         </is>
       </c>
-      <c r="B12" s="12">
+      <c r="B12" s="13">
         <f>B8/(B8+B9)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>债务权重</t>
         </is>
       </c>
-      <c r="B13" s="12">
+      <c r="B13" s="13">
         <f>B9/(B8+B9)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>WACC</t>
         </is>
       </c>
-      <c r="B14" s="12">
+      <c r="B14" s="13">
         <f>B13*B10+B14*B11</f>
         <v/>
       </c>
@@ -1602,22 +1629,22 @@
           <t>营业总收入</t>
         </is>
       </c>
-      <c r="B3" s="8" t="n">
+      <c r="B3" s="9" t="n">
         <v>2857.09729</v>
       </c>
-      <c r="C3" s="8" t="n">
+      <c r="C3" s="9" t="n">
         <v>3433.60825</v>
       </c>
-      <c r="D3" s="8" t="n">
+      <c r="D3" s="9" t="n">
         <v>3457.08706</v>
       </c>
-      <c r="E3" s="8" t="n">
+      <c r="E3" s="9" t="n">
         <v>3737.09804</v>
       </c>
-      <c r="F3" s="8" t="n">
+      <c r="F3" s="9" t="n">
         <v>4090.84266</v>
       </c>
-      <c r="G3" s="8" t="n">
+      <c r="G3" s="9" t="n">
         <v>4585.02407</v>
       </c>
     </row>
@@ -1627,20 +1654,20 @@
           <t>收入增速</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n"/>
-      <c r="C4" s="12" t="n">
+      <c r="B4" s="13" t="n"/>
+      <c r="C4" s="13" t="n">
         <v>0.2017820541210902</v>
       </c>
-      <c r="D4" s="12" t="n">
+      <c r="D4" s="13" t="n">
         <v>0.006837940816340815</v>
       </c>
-      <c r="E4" s="12" t="n">
+      <c r="E4" s="13" t="n">
         <v>0.08099621882244423</v>
       </c>
-      <c r="F4" s="12" t="n">
+      <c r="F4" s="13" t="n">
         <v>0.09465757018245102</v>
       </c>
-      <c r="G4" s="12" t="n">
+      <c r="G4" s="13" t="n">
         <v>0.1208018618833901</v>
       </c>
     </row>
@@ -1650,22 +1677,22 @@
           <t>毛利率</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
+      <c r="B5" s="13" t="n">
         <v>0.2359836895858733</v>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="13" t="n">
         <v>0.2234011669793722</v>
       </c>
-      <c r="D5" s="12" t="n">
+      <c r="D5" s="13" t="n">
         <v>0.2411823264873174</v>
       </c>
-      <c r="E5" s="12" t="n">
+      <c r="E5" s="13" t="n">
         <v>0.2558880579970014</v>
       </c>
-      <c r="F5" s="12" t="n">
+      <c r="F5" s="13" t="n">
         <v>0.2629401175747004</v>
       </c>
-      <c r="G5" s="12" t="n">
+      <c r="G5" s="13" t="n">
         <v>0.262729706891157</v>
       </c>
     </row>
@@ -1675,22 +1702,22 @@
           <t>EBIT</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="9" t="n">
         <v>293.06102</v>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C6" s="9" t="n">
         <v>298.9345</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="9" t="n">
         <v>309.4913299999999</v>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="9" t="n">
         <v>361.33821</v>
       </c>
-      <c r="F6" s="8" t="n">
+      <c r="F6" s="9" t="n">
         <v>419.42116</v>
       </c>
-      <c r="G6" s="8" t="n">
+      <c r="G6" s="9" t="n">
         <v>468.5237299999999</v>
       </c>
     </row>
@@ -1700,22 +1727,22 @@
           <t>EBIT 利润率</t>
         </is>
       </c>
-      <c r="B7" s="12" t="n">
+      <c r="B7" s="13" t="n">
         <v>0.102572992885377</v>
       </c>
-      <c r="C7" s="12" t="n">
+      <c r="C7" s="13" t="n">
         <v>0.08706132972507856</v>
       </c>
-      <c r="D7" s="12" t="n">
+      <c r="D7" s="13" t="n">
         <v>0.08952373042060444</v>
       </c>
-      <c r="E7" s="12" t="n">
+      <c r="E7" s="13" t="n">
         <v>0.09668951847995939</v>
       </c>
-      <c r="F7" s="12" t="n">
+      <c r="F7" s="13" t="n">
         <v>0.1025268373435805</v>
       </c>
-      <c r="G7" s="12" t="n">
+      <c r="G7" s="13" t="n">
         <v>0.1021856642074291</v>
       </c>
     </row>
@@ -1725,22 +1752,22 @@
           <t>有效税率</t>
         </is>
       </c>
-      <c r="B8" s="12" t="n">
+      <c r="B8" s="13" t="n">
         <v>0.1312865564395692</v>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="13" t="n">
         <v>0.1394576069953375</v>
       </c>
-      <c r="D8" s="12" t="n">
+      <c r="D8" s="13" t="n">
         <v>0.1472053483570499</v>
       </c>
-      <c r="E8" s="12" t="n">
+      <c r="E8" s="13" t="n">
         <v>0.1621715759871171</v>
       </c>
-      <c r="F8" s="12" t="n">
+      <c r="F8" s="13" t="n">
         <v>0.1698988039043948</v>
       </c>
-      <c r="G8" s="12" t="n">
+      <c r="G8" s="13" t="n">
         <v>0.1613467393438524</v>
       </c>
     </row>
@@ -1750,22 +1777,22 @@
           <t>归母净利润</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n">
+      <c r="B9" s="9" t="n">
         <v>272.22969</v>
       </c>
-      <c r="C9" s="8" t="n">
+      <c r="C9" s="9" t="n">
         <v>285.7365</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="9" t="n">
         <v>295.53507</v>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="9" t="n">
         <v>337.19935</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="F9" s="9" t="n">
         <v>385.37237</v>
       </c>
-      <c r="G9" s="8" t="n">
+      <c r="G9" s="9" t="n">
         <v>439.45411</v>
       </c>
     </row>
@@ -1775,22 +1802,22 @@
           <t>ROE</t>
         </is>
       </c>
-      <c r="B10" s="12" t="n">
+      <c r="B10" s="13" t="n">
         <v>0.2316527857506697</v>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="13" t="n">
         <v>0.228830618132775</v>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="D10" s="13" t="n">
         <v>0.2067615224002569</v>
       </c>
-      <c r="E10" s="12" t="n">
+      <c r="E10" s="13" t="n">
         <v>0.2070246700269356</v>
       </c>
-      <c r="F10" s="12" t="n">
+      <c r="F10" s="13" t="n">
         <v>0.1777957410179597</v>
       </c>
-      <c r="G10" s="12" t="n">
+      <c r="G10" s="13" t="n">
         <v>0.1968692504508026</v>
       </c>
     </row>
@@ -1800,22 +1827,22 @@
           <t>经营现金流</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n">
+      <c r="B11" s="9" t="n">
         <v>295.57117</v>
       </c>
-      <c r="C11" s="8" t="n">
+      <c r="C11" s="9" t="n">
         <v>350.91704</v>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="9" t="n">
         <v>346.57828</v>
       </c>
-      <c r="E11" s="8" t="n">
+      <c r="E11" s="9" t="n">
         <v>579.02611</v>
       </c>
-      <c r="F11" s="8" t="n">
+      <c r="F11" s="9" t="n">
         <v>605.11572</v>
       </c>
-      <c r="G11" s="8" t="n">
+      <c r="G11" s="9" t="n">
         <v>533.4593</v>
       </c>
     </row>
@@ -1825,22 +1852,22 @@
           <t>经营现金流 / 归母净利润</t>
         </is>
       </c>
-      <c r="B12" s="12" t="n">
+      <c r="B12" s="13" t="n">
         <v>1.085741860118197</v>
       </c>
-      <c r="C12" s="12" t="n">
+      <c r="C12" s="13" t="n">
         <v>1.228114154124517</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="13" t="n">
         <v>1.17271456142244</v>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="13" t="n">
         <v>1.71716259239527</v>
       </c>
-      <c r="F12" s="12" t="n">
+      <c r="F12" s="13" t="n">
         <v>1.570210443473153</v>
       </c>
-      <c r="G12" s="12" t="n">
+      <c r="G12" s="13" t="n">
         <v>1.213913552884964</v>
       </c>
     </row>
@@ -1850,22 +1877,22 @@
           <t>折旧摊销 / 收入</t>
         </is>
       </c>
-      <c r="B13" s="12" t="n">
+      <c r="B13" s="13" t="n">
         <v>0.01757117623390416</v>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="13" t="n">
         <v>0.01800686493574216</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="13" t="n">
         <v>0.01882486581058216</v>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="13" t="n">
         <v>0.01966477978725974</v>
       </c>
-      <c r="F13" s="12" t="n">
+      <c r="F13" s="13" t="n">
         <v>0.01912525279082721</v>
       </c>
-      <c r="G13" s="12" t="n">
+      <c r="G13" s="13" t="n">
         <v>0.02037000211429642</v>
       </c>
     </row>
@@ -1875,22 +1902,22 @@
           <t>资本开支 / 收入</t>
         </is>
       </c>
-      <c r="B14" s="12" t="n">
+      <c r="B14" s="13" t="n">
         <v>0.01629829693338864</v>
       </c>
-      <c r="C14" s="12" t="n">
+      <c r="C14" s="13" t="n">
         <v>0.01987808888797957</v>
       </c>
-      <c r="D14" s="12" t="n">
+      <c r="D14" s="13" t="n">
         <v>0.0212667915860933</v>
       </c>
-      <c r="E14" s="12" t="n">
+      <c r="E14" s="13" t="n">
         <v>0.01689559902474488</v>
       </c>
-      <c r="F14" s="12" t="n">
+      <c r="F14" s="13" t="n">
         <v>0.01916386586229645</v>
       </c>
-      <c r="G14" s="12" t="n">
+      <c r="G14" s="13" t="n">
         <v>0.02430061179591583</v>
       </c>
     </row>
@@ -1900,23 +1927,23 @@
           <t>营运资本 / 收入</t>
         </is>
       </c>
-      <c r="B15" s="12" t="n">
-        <v>-0.1249210173028444</v>
-      </c>
-      <c r="C15" s="12" t="n">
-        <v>-0.05071215098577422</v>
-      </c>
-      <c r="D15" s="12" t="n">
-        <v>0.02491387648189572</v>
-      </c>
-      <c r="E15" s="12" t="n">
-        <v>-0.08057666316937193</v>
-      </c>
-      <c r="F15" s="12" t="n">
-        <v>-0.09638884278184388</v>
-      </c>
-      <c r="G15" s="12" t="n">
-        <v>0.0808002323093584</v>
+      <c r="B15" s="13" t="n">
+        <v>-0.1191145506984118</v>
+      </c>
+      <c r="C15" s="13" t="n">
+        <v>-0.1217260821760898</v>
+      </c>
+      <c r="D15" s="13" t="n">
+        <v>-0.08226443102650705</v>
+      </c>
+      <c r="E15" s="13" t="n">
+        <v>-0.1179968936538791</v>
+      </c>
+      <c r="F15" s="13" t="n">
+        <v>-0.1288111799440363</v>
+      </c>
+      <c r="G15" s="13" t="n">
+        <v>-0.1354150775483279</v>
       </c>
     </row>
     <row r="16">
@@ -1925,21 +1952,21 @@
           <t>FCFF</t>
         </is>
       </c>
-      <c r="B16" s="8" t="n"/>
-      <c r="C16" s="8" t="n">
-        <v>68.03491998165237</v>
-      </c>
-      <c r="D16" s="8" t="n">
-        <v>-4.764499046136763</v>
-      </c>
-      <c r="E16" s="8" t="n">
-        <v>700.3404530199361</v>
-      </c>
-      <c r="F16" s="8" t="n">
-        <v>441.1927465838063</v>
-      </c>
-      <c r="G16" s="8" t="n">
-        <v>-389.8755861407195</v>
+      <c r="B16" s="9" t="n"/>
+      <c r="C16" s="9" t="n">
+        <v>328.4585799816523</v>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>121.9262209538633</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>469.6587830199361</v>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>433.9843565838063</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>468.8421338592805</v>
       </c>
     </row>
     <row r="17">
@@ -1948,22 +1975,22 @@
           <t>现金</t>
         </is>
       </c>
-      <c r="B17" s="8" t="n">
+      <c r="B17" s="9" t="n">
         <v>1094.50083</v>
       </c>
-      <c r="C17" s="8" t="n">
+      <c r="C17" s="9" t="n">
         <v>777.54758</v>
       </c>
-      <c r="D17" s="8" t="n">
+      <c r="D17" s="9" t="n">
         <v>585.54692</v>
       </c>
-      <c r="E17" s="8" t="n">
+      <c r="E17" s="9" t="n">
         <v>834.6443400000001</v>
       </c>
-      <c r="F17" s="8" t="n">
+      <c r="F17" s="9" t="n">
         <v>1473.46421</v>
       </c>
-      <c r="G17" s="8" t="n">
+      <c r="G17" s="9" t="n">
         <v>859.57867</v>
       </c>
     </row>
@@ -1973,22 +2000,22 @@
           <t>有息负债</t>
         </is>
       </c>
-      <c r="B18" s="8" t="n">
+      <c r="B18" s="9" t="n">
         <v>590.81397</v>
       </c>
-      <c r="C18" s="8" t="n">
+      <c r="C18" s="9" t="n">
         <v>555.96735</v>
       </c>
-      <c r="D18" s="8" t="n">
+      <c r="D18" s="9" t="n">
         <v>677.6715</v>
       </c>
-      <c r="E18" s="8" t="n">
+      <c r="E18" s="9" t="n">
         <v>746.8090999999999</v>
       </c>
-      <c r="F18" s="8" t="n">
+      <c r="F18" s="9" t="n">
         <v>862.55072</v>
       </c>
-      <c r="G18" s="8" t="n">
+      <c r="G18" s="9" t="n">
         <v>674.80997</v>
       </c>
     </row>

</xml_diff>